<commit_message>
second admin module done
</commit_message>
<xml_diff>
--- a/orengeHRM/xldata/Generate_report_orenge.xlsx
+++ b/orengeHRM/xldata/Generate_report_orenge.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="113">
   <si>
     <t>Testcases id</t>
   </si>
@@ -50,7 +50,7 @@
     <t>Applicationlogin</t>
   </si>
   <si>
-    <t>Y</t>
+    <t>N</t>
   </si>
   <si>
     <t>TC002</t>
@@ -59,13 +59,16 @@
     <t>Admin</t>
   </si>
   <si>
+    <t>y</t>
+  </si>
+  <si>
     <t>TC003</t>
   </si>
   <si>
     <t>PIM</t>
   </si>
   <si>
-    <t>N</t>
+    <t>n</t>
   </si>
   <si>
     <t>Description</t>
@@ -206,13 +209,13 @@
     <t>systemUser_userName</t>
   </si>
   <si>
-    <t>varafdfhdtlq</t>
+    <t>vafhsddsf</t>
   </si>
   <si>
     <t xml:space="preserve">wait for Status </t>
   </si>
   <si>
-    <t>systemUser[status]</t>
+    <t>//select[@id='systemUser_status']</t>
   </si>
   <si>
     <t xml:space="preserve">select the Status </t>
@@ -239,16 +242,22 @@
     <t>btnSave</t>
   </si>
   <si>
+    <t>wait for save button</t>
+  </si>
+  <si>
+    <t>//input[@id='btnSave']</t>
+  </si>
+  <si>
     <t>wait for username searchbutton</t>
   </si>
   <si>
-    <t>searchSystemUser_userName</t>
+    <t>click on username</t>
   </si>
   <si>
     <t>enter the username</t>
   </si>
   <si>
-    <t>varafdfhdt1</t>
+    <t>//input[@id='searchSystemUser_userName']</t>
   </si>
   <si>
     <t>click on search</t>
@@ -269,6 +278,87 @@
     <t>verifyusernametable</t>
   </si>
   <si>
+    <t>wait for PIM menu</t>
+  </si>
+  <si>
+    <t>//b[normalize-space()='PIM']</t>
+  </si>
+  <si>
+    <t>click on PIM</t>
+  </si>
+  <si>
+    <t>wait for add button</t>
+  </si>
+  <si>
+    <t>//input[@name='btnAdd']</t>
+  </si>
+  <si>
+    <t>enter the firstname</t>
+  </si>
+  <si>
+    <t>//input[@name='firstName']</t>
+  </si>
+  <si>
+    <t>uday</t>
+  </si>
+  <si>
+    <t>enter the midname</t>
+  </si>
+  <si>
+    <t>//input[@id='middleName']</t>
+  </si>
+  <si>
+    <t>k</t>
+  </si>
+  <si>
+    <t>enter the lastname</t>
+  </si>
+  <si>
+    <t>//input[@id='lastName']</t>
+  </si>
+  <si>
+    <t>varm</t>
+  </si>
+  <si>
+    <t>captureemployeid</t>
+  </si>
+  <si>
+    <t>employeeId</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wait for some time </t>
+  </si>
+  <si>
+    <t>//input[@id='photofile']</t>
+  </si>
+  <si>
+    <t>select the file location</t>
+  </si>
+  <si>
+    <t>UploadFile</t>
+  </si>
+  <si>
+    <t>C:/Users/DELL/Downloads/Hybridstructure_lyst1750226921116 (2).text'</t>
+  </si>
+  <si>
+    <t>click on save button</t>
+  </si>
+  <si>
+    <t>wait for emplottable</t>
+  </si>
+  <si>
+    <t>verify the employid</t>
+  </si>
+  <si>
+    <t>employtable</t>
+  </si>
+  <si>
+    <t>//*[@id='resultTable']/tbody/tr[1]/td[2]/a</t>
+  </si>
+  <si>
+    <t>Blocked</t>
+  </si>
+  <si>
     <t>Pass</t>
   </si>
   <si>
@@ -279,9 +369,6 @@
   </si>
   <si>
     <t>FAIL</t>
-  </si>
-  <si>
-    <t>Blocked</t>
   </si>
 </sst>
 </file>
@@ -294,7 +381,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="102">
+  <fonts count="82">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -311,6 +398,12 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="9"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Courier New"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF800080"/>
@@ -754,111 +847,6 @@
       <sz val="11.0"/>
       <b val="true"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
   </fonts>
   <fills count="40">
     <fill>
@@ -1061,6 +1049,16 @@
     </fill>
     <fill>
       <patternFill patternType="none">
+        <fgColor indexed="12"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor indexed="12"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="none">
         <fgColor indexed="17"/>
       </patternFill>
     </fill>
@@ -1077,16 +1075,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="10"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="none">
-        <fgColor indexed="12"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="12"/>
       </patternFill>
     </fill>
   </fills>
@@ -1231,137 +1219,137 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1374,93 +1362,75 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" quotePrefix="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="23" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="25" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="26" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="27" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="28" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="29" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="30" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="31" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="32" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="33" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="34" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="35" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="36" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="37" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="38" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="39" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="40" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="41" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="42" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="43" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="44" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="45" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="46" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="47" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="48" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="49" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="50" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="51" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="52" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="53" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="54" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="55" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="56" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="57" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="58" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="59" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="60" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="61" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="62" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="63" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="64" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="23" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="24" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="25" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="26" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="27" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="28" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="29" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="30" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="31" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="32" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="33" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="34" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="35" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="36" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="37" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="38" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="39" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="40" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="41" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="42" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="43" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="44" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="45" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="46" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="47" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="48" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="49" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="50" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="51" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="52" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="53" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="54" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="55" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="56" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="57" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="58" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="59" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="60" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="61" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="62" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="63" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="64" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
     <xf numFmtId="0" fontId="65" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="66" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="66" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
     <xf numFmtId="0" fontId="67" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="68" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="69" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="68" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="69" fillId="39" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
     <xf numFmtId="0" fontId="70" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="71" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="72" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="71" fillId="39" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="72" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
     <xf numFmtId="0" fontId="73" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="74" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="75" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="74" fillId="39" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="75" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
     <xf numFmtId="0" fontId="76" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="77" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="78" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="77" fillId="39" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="78" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
     <xf numFmtId="0" fontId="79" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="80" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="80" fillId="39" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
     <xf numFmtId="0" fontId="81" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="82" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="83" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="84" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="85" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="86" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="87" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="88" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="89" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="90" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="91" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="92" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="93" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="94" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="95" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="96" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="97" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="98" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="99" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="100" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="101" fillId="39" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2034,8 +2004,8 @@
       <c r="C2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="D2" t="s" s="23">
-        <v>80</v>
+      <c r="D2" t="s" s="7">
+        <v>108</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2046,24 +2016,24 @@
         <v>8</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D3" t="s" s="85">
-        <v>82</v>
+        <v>9</v>
+      </c>
+      <c r="D3" t="s" s="65">
+        <v>112</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="D4" t="s" s="86">
-        <v>83</v>
+        <v>12</v>
+      </c>
+      <c r="D4" t="s" s="66">
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -2087,203 +2057,185 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="18.75" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" t="s" s="6">
-        <v>79</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="F2" s="3"/>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" t="s" s="8">
-        <v>79</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="F3" s="3"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F4" t="s" s="10">
-        <v>79</v>
-      </c>
+      <c r="F4" s="3"/>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F5" t="s" s="12">
-        <v>79</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="F5" s="3"/>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E6" s="3">
         <v>3000</v>
       </c>
-      <c r="F6" t="s" s="14">
-        <v>79</v>
-      </c>
+      <c r="F6" s="3"/>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F7" t="s" s="16">
-        <v>79</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="F7" s="3"/>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E8" s="3">
         <v>3000</v>
       </c>
-      <c r="F8" t="s" s="18">
-        <v>79</v>
-      </c>
+      <c r="F8" s="3"/>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="F9" t="s" s="20">
-        <v>79</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="F9" s="3"/>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F10" t="s" s="22">
-        <v>79</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="F10" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2294,7 +2246,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="27.5714285714286"/>
@@ -2306,462 +2258,462 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="18.75" spans="1:6">
       <c r="A1" s="2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" t="s" s="24">
-        <v>79</v>
+        <v>21</v>
+      </c>
+      <c r="F2" t="s" s="8">
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" t="s" s="26">
-        <v>79</v>
+        <v>21</v>
+      </c>
+      <c r="F3" t="s" s="10">
+        <v>109</v>
       </c>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F4" t="s" s="28">
-        <v>79</v>
+      <c r="F4" t="s" s="12">
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F5" t="s" s="30">
-        <v>79</v>
+        <v>30</v>
+      </c>
+      <c r="F5" t="s" s="14">
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F6" t="s" s="32">
-        <v>79</v>
+        <v>21</v>
+      </c>
+      <c r="F6" t="s" s="16">
+        <v>109</v>
       </c>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>38</v>
-      </c>
-      <c r="F7" t="s" s="34">
-        <v>79</v>
+        <v>39</v>
+      </c>
+      <c r="F7" t="s" s="18">
+        <v>109</v>
       </c>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E8" s="3">
         <v>10</v>
       </c>
-      <c r="F8" t="s" s="36">
-        <v>79</v>
+      <c r="F8" t="s" s="20">
+        <v>109</v>
       </c>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>45</v>
-      </c>
       <c r="E9" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F9" t="s" s="38">
-        <v>79</v>
+        <v>21</v>
+      </c>
+      <c r="F9" t="s" s="22">
+        <v>109</v>
       </c>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F10" t="s" s="40">
-        <v>79</v>
+        <v>21</v>
+      </c>
+      <c r="F10" t="s" s="24">
+        <v>109</v>
       </c>
     </row>
     <row r="11" customFormat="1" spans="1:6">
       <c r="A11" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E11" s="3">
         <v>10</v>
       </c>
-      <c r="F11" t="s" s="42">
-        <v>79</v>
+      <c r="F11" t="s" s="26">
+        <v>109</v>
       </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>51</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>50</v>
       </c>
       <c r="E12" s="3">
         <v>0</v>
       </c>
-      <c r="F12" t="s" s="44">
-        <v>79</v>
+      <c r="F12" t="s" s="28">
+        <v>109</v>
       </c>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="F13" t="s" s="46">
-        <v>79</v>
+        <v>56</v>
+      </c>
+      <c r="F13" t="s" s="30">
+        <v>109</v>
       </c>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="F14" t="s" s="48">
-        <v>79</v>
+        <v>59</v>
+      </c>
+      <c r="F14" t="s" s="32">
+        <v>109</v>
       </c>
     </row>
     <row r="15" customFormat="1" spans="1:6">
-      <c r="A15" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>43</v>
+      <c r="A15" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>44</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E15" s="3">
         <v>10</v>
       </c>
-      <c r="F15" t="s" s="50">
-        <v>81</v>
+      <c r="F15" t="s" s="34">
+        <v>109</v>
       </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>61</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>60</v>
       </c>
       <c r="E16" s="3">
         <v>0</v>
       </c>
-      <c r="F16" t="s" s="53">
-        <v>79</v>
+      <c r="F16" t="s" s="36">
+        <v>109</v>
       </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F17" t="s" s="56">
-        <v>79</v>
+        <v>30</v>
+      </c>
+      <c r="F17" t="s" s="38">
+        <v>109</v>
       </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="F18" t="s" s="59">
-        <v>79</v>
+        <v>30</v>
+      </c>
+      <c r="F18" t="s" s="40">
+        <v>109</v>
       </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E19" s="4">
+        <v>21</v>
+      </c>
+      <c r="E19" s="3">
         <v>3000</v>
       </c>
-      <c r="F19" t="s" s="62">
-        <v>79</v>
+      <c r="F19" t="s" s="42">
+        <v>109</v>
       </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F20" t="s" s="65">
-        <v>79</v>
+        <v>21</v>
+      </c>
+      <c r="F20" t="s" s="44">
+        <v>109</v>
       </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B21" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B21" s="3" t="s">
-        <v>33</v>
-      </c>
       <c r="C21" s="3" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F21" t="s" s="68">
-        <v>79</v>
+        <v>71</v>
+      </c>
+      <c r="E21" s="3">
+        <v>3000</v>
+      </c>
+      <c r="F21" t="s" s="46">
+        <v>109</v>
       </c>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="3" t="s">
+        <v>68</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D22" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B22" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E22" s="3">
-        <v>2000</v>
-      </c>
-      <c r="F22" t="s" s="71">
-        <v>79</v>
+      <c r="E22" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F22" t="s" s="48">
+        <v>109</v>
       </c>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>24</v>
+        <v>44</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="F23" t="s" s="74">
-        <v>81</v>
+        <v>58</v>
+      </c>
+      <c r="E23" s="3">
+        <v>10</v>
+      </c>
+      <c r="F23" t="s" s="50">
+        <v>109</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -2769,59 +2721,99 @@
         <v>73</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="F24" t="s" s="77">
-        <v>81</v>
+        <v>21</v>
+      </c>
+      <c r="F24" t="s" s="52">
+        <v>109</v>
       </c>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D25" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="B25" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="E25" s="3">
-        <v>10</v>
-      </c>
-      <c r="F25" t="s" s="80">
-        <v>81</v>
+      <c r="E25" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F25" t="s" s="54">
+        <v>111</v>
       </c>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D26" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="E26" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F26" t="s" s="57">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6">
+      <c r="A27" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="B27" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="D26" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="F26" t="s" s="83">
+      <c r="C27" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>79</v>
+      </c>
+      <c r="E27" s="3">
+        <v>10</v>
+      </c>
+      <c r="F27" t="s" s="60">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6">
+      <c r="A28" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F28" t="s" s="63">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -2833,9 +2825,362 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
-  <sheetData/>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <cols>
+    <col min="1" max="1" customWidth="true" width="26.4285714285714"/>
+    <col min="2" max="2" customWidth="true" width="26.2857142857143"/>
+    <col min="3" max="3" customWidth="true" width="15.5714285714286"/>
+    <col min="4" max="4" customWidth="true" width="33.8571428571429"/>
+    <col min="5" max="5" customWidth="true" width="70.1428571428571"/>
+    <col min="6" max="6" customWidth="true" width="12.5714285714286"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="1" customFormat="1" ht="18.75" spans="1:6">
+      <c r="A1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="3"/>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" s="3"/>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="3"/>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="3"/>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E7" s="3">
+        <v>10</v>
+      </c>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="3"/>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E9" s="3">
+        <v>10</v>
+      </c>
+      <c r="F9" s="3"/>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F10" s="3"/>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="F11" s="3"/>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="F12" s="3"/>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>94</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="F13" s="3"/>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F14" s="3"/>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="E15" s="3">
+        <v>5000</v>
+      </c>
+      <c r="F15" s="3"/>
+    </row>
+    <row r="16" spans="1:6">
+      <c r="A16" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>101</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="F16" s="3"/>
+    </row>
+    <row r="17" spans="1:6">
+      <c r="A17" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F17" s="3"/>
+    </row>
+    <row r="18" spans="1:6">
+      <c r="A18" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F18" s="3"/>
+    </row>
+    <row r="19" spans="1:6">
+      <c r="A19" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>106</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>107</v>
+      </c>
+      <c r="E19" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F19" s="3"/>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>

</xml_diff>

<commit_message>
recurment module pending for calander only
</commit_message>
<xml_diff>
--- a/orengeHRM/xldata/Generate_report_orenge.xlsx
+++ b/orengeHRM/xldata/Generate_report_orenge.xlsx
@@ -4,13 +4,14 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7620" activeTab="2"/>
+    <workbookView windowWidth="20490" windowHeight="7620"/>
   </bookViews>
   <sheets>
     <sheet name="masterTestcases" sheetId="1" r:id="rId1"/>
     <sheet name="Applicationlogin" sheetId="2" r:id="rId2"/>
     <sheet name="Admin" sheetId="3" r:id="rId3"/>
     <sheet name="PIM" sheetId="4" r:id="rId4"/>
+    <sheet name="Recruitment" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -30,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="347" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="466" uniqueCount="133">
   <si>
     <t>Testcases id</t>
   </si>
@@ -59,18 +60,21 @@
     <t>Admin</t>
   </si>
   <si>
+    <t>TC003</t>
+  </si>
+  <si>
+    <t>PIM</t>
+  </si>
+  <si>
+    <t>TC004</t>
+  </si>
+  <si>
+    <t>Recruitment</t>
+  </si>
+  <si>
     <t>y</t>
   </si>
   <si>
-    <t>TC003</t>
-  </si>
-  <si>
-    <t>PIM</t>
-  </si>
-  <si>
-    <t>n</t>
-  </si>
-  <si>
     <t>Description</t>
   </si>
   <si>
@@ -209,7 +213,7 @@
     <t>systemUser_userName</t>
   </si>
   <si>
-    <t>vafhsddsf</t>
+    <t>uday121l</t>
   </si>
   <si>
     <t xml:space="preserve">wait for Status </t>
@@ -239,45 +243,36 @@
     <t>click on the savebutton</t>
   </si>
   <si>
-    <t>btnSave</t>
+    <t>//input[@id='btnSave']</t>
   </si>
   <si>
     <t>wait for save button</t>
   </si>
   <si>
-    <t>//input[@id='btnSave']</t>
-  </si>
-  <si>
-    <t>wait for username searchbutton</t>
-  </si>
-  <si>
-    <t>click on username</t>
+    <t>wait for the username</t>
+  </si>
+  <si>
+    <t>//input[@name='searchSystemUser[userName]']</t>
   </si>
   <si>
     <t>enter the username</t>
   </si>
   <si>
-    <t>//input[@id='searchSystemUser_userName']</t>
-  </si>
-  <si>
-    <t>click on search</t>
+    <t>click on the search button</t>
   </si>
   <si>
     <t>//input[@id='searchBtn']</t>
   </si>
   <si>
-    <t>wait for usernamein table</t>
+    <t>verify the usernamein table</t>
+  </si>
+  <si>
+    <t>verifyusernametable</t>
   </si>
   <si>
     <t>//table[@id='resultTable']/tbody/tr[1]/td[2]</t>
   </si>
   <si>
-    <t>verify the usernamein table</t>
-  </si>
-  <si>
-    <t>verifyusernametable</t>
-  </si>
-  <si>
     <t>wait for PIM menu</t>
   </si>
   <si>
@@ -332,15 +327,6 @@
     <t>//input[@id='photofile']</t>
   </si>
   <si>
-    <t>select the file location</t>
-  </si>
-  <si>
-    <t>UploadFile</t>
-  </si>
-  <si>
-    <t>C:/Users/DELL/Downloads/Hybridstructure_lyst1750226921116 (2).text'</t>
-  </si>
-  <si>
     <t>click on save button</t>
   </si>
   <si>
@@ -356,6 +342,87 @@
     <t>//*[@id='resultTable']/tbody/tr[1]/td[2]/a</t>
   </si>
   <si>
+    <t>wait for Recruitment</t>
+  </si>
+  <si>
+    <t>//b[normalize-space()='Recruitment']</t>
+  </si>
+  <si>
+    <t>clikck on the recruitment</t>
+  </si>
+  <si>
+    <t>//input[@id='btnAdd']</t>
+  </si>
+  <si>
+    <t>wait for firstname</t>
+  </si>
+  <si>
+    <t>//input[@id='addCandidate_firstName']</t>
+  </si>
+  <si>
+    <t>//input[@id='addCandidate_middleName']</t>
+  </si>
+  <si>
+    <t>//input[@id='addCandidate_lastName']</t>
+  </si>
+  <si>
+    <t>varaa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">wait for email id </t>
+  </si>
+  <si>
+    <t>//input[@id='addCandidate_email']</t>
+  </si>
+  <si>
+    <t>enter the emailid</t>
+  </si>
+  <si>
+    <t>ydaa@gmail.com</t>
+  </si>
+  <si>
+    <t>wait for  contact</t>
+  </si>
+  <si>
+    <t>//input[@id='addCandidate_contactNo']</t>
+  </si>
+  <si>
+    <t>enter the contact number</t>
+  </si>
+  <si>
+    <t>enter the keypad</t>
+  </si>
+  <si>
+    <t>//input[@id='addCandidate_keyWords']</t>
+  </si>
+  <si>
+    <t>udaa</t>
+  </si>
+  <si>
+    <t>enter the comments</t>
+  </si>
+  <si>
+    <t>//textarea[@id='addCandidate_comment']</t>
+  </si>
+  <si>
+    <t>its working fine</t>
+  </si>
+  <si>
+    <t>select the datacalander</t>
+  </si>
+  <si>
+    <t>selectcalander</t>
+  </si>
+  <si>
+    <t>//input[@id='addCandidate_appliedDate']</t>
+  </si>
+  <si>
+    <t xml:space="preserve">click on checkbox </t>
+  </si>
+  <si>
+    <t>//input[@id='addCandidate_consentToKeepData']</t>
+  </si>
+  <si>
     <t>Blocked</t>
   </si>
   <si>
@@ -363,12 +430,6 @@
   </si>
   <si>
     <t>PASS</t>
-  </si>
-  <si>
-    <t>Fail</t>
-  </si>
-  <si>
-    <t>FAIL</t>
   </si>
 </sst>
 </file>
@@ -381,7 +442,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="82">
+  <fonts count="73">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -395,6 +456,14 @@
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -412,14 +481,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
@@ -802,53 +863,8 @@
       <sz val="11.0"/>
       <b val="true"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="11.0"/>
-      <b val="true"/>
-    </font>
   </fonts>
-  <fills count="40">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1065,16 +1081,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="17"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="none">
-        <fgColor indexed="10"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor indexed="10"/>
       </patternFill>
     </fill>
   </fills>
@@ -1219,12 +1225,12 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
@@ -1349,7 +1355,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="67">
+  <cellXfs count="58">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1362,18 +1368,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" quotePrefix="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="6" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="23" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="24" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="23" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="24" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
     <xf numFmtId="0" fontId="25" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
     <xf numFmtId="0" fontId="26" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
     <xf numFmtId="0" fontId="27" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
@@ -1418,19 +1424,10 @@
     <xf numFmtId="0" fontId="66" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
     <xf numFmtId="0" fontId="67" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
     <xf numFmtId="0" fontId="68" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="69" fillId="39" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="69" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
     <xf numFmtId="0" fontId="70" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="71" fillId="39" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
+    <xf numFmtId="0" fontId="71" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
     <xf numFmtId="0" fontId="72" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="73" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="74" fillId="39" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="75" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="76" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="77" fillId="39" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="78" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="79" fillId="37" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="80" fillId="39" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
-    <xf numFmtId="0" fontId="81" fillId="35" borderId="0" xfId="0" applyFill="true" applyFont="true"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1971,8 +1968,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="3" outlineLevelCol="3"/>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="4" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="24.0"/>
     <col min="2" max="2" customWidth="true" width="28.8571428571429"/>
@@ -2005,7 +2002,7 @@
         <v>6</v>
       </c>
       <c r="D2" t="s" s="7">
-        <v>108</v>
+        <v>130</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -2016,24 +2013,38 @@
         <v>8</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s" s="65">
-        <v>112</v>
+        <v>6</v>
+      </c>
+      <c r="D3" t="s" s="8">
+        <v>130</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="C4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4" t="s" s="9">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="B5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="D4" t="s" s="66">
-        <v>108</v>
+      <c r="C5" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="s" s="57">
+        <v>132</v>
       </c>
     </row>
   </sheetData>
@@ -2057,72 +2068,72 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="18.75" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F2" s="3"/>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F3" s="3"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>8</v>
@@ -2131,34 +2142,34 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F5" s="3"/>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E6" s="3">
         <v>3000</v>
@@ -2167,34 +2178,34 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F7" s="3"/>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E8" s="3">
         <v>3000</v>
@@ -2203,37 +2214,37 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F9" s="3"/>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F10" s="3"/>
     </row>
@@ -2258,563 +2269,509 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="18.75" spans="1:6">
       <c r="A1" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F2" t="s" s="8">
-        <v>109</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="F2" s="3"/>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F3" t="s" s="10">
-        <v>109</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="F3" s="3"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F4" t="s" s="12">
-        <v>109</v>
-      </c>
+      <c r="F4" s="3"/>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" t="s" s="14">
-        <v>109</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="F5" s="3"/>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F6" t="s" s="16">
-        <v>109</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="F6" s="3"/>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="F7" t="s" s="18">
-        <v>109</v>
-      </c>
+        <v>40</v>
+      </c>
+      <c r="F7" s="3"/>
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E8" s="3">
         <v>10</v>
       </c>
-      <c r="F8" t="s" s="20">
-        <v>109</v>
-      </c>
+      <c r="F8" s="3"/>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B9" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>46</v>
-      </c>
       <c r="E9" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F9" t="s" s="22">
-        <v>109</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="F9" s="3"/>
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F10" t="s" s="24">
-        <v>109</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="F10" s="3"/>
     </row>
     <row r="11" customFormat="1" spans="1:6">
       <c r="A11" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E11" s="3">
         <v>10</v>
       </c>
-      <c r="F11" t="s" s="26">
-        <v>109</v>
-      </c>
+      <c r="F11" s="3"/>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>52</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>51</v>
       </c>
       <c r="E12" s="3">
         <v>0</v>
       </c>
-      <c r="F12" t="s" s="28">
-        <v>109</v>
-      </c>
+      <c r="F12" s="3"/>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F13" t="s" s="30">
-        <v>109</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="F13" s="3"/>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="F14" t="s" s="32">
-        <v>109</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="F14" s="3"/>
     </row>
     <row r="15" customFormat="1" spans="1:6">
       <c r="A15" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E15" s="3">
         <v>10</v>
       </c>
-      <c r="F15" t="s" s="34">
-        <v>109</v>
-      </c>
+      <c r="F15" s="3"/>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>62</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>61</v>
       </c>
       <c r="E16" s="3">
         <v>0</v>
       </c>
-      <c r="F16" t="s" s="36">
-        <v>109</v>
-      </c>
+      <c r="F16" s="3"/>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="F17" t="s" s="38">
-        <v>109</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F17" s="3"/>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="F18" t="s" s="40">
-        <v>109</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F18" s="3"/>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E19" s="3">
         <v>3000</v>
       </c>
-      <c r="F19" t="s" s="42">
-        <v>109</v>
-      </c>
+      <c r="F19" s="3"/>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F20" t="s" s="44">
-        <v>109</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="F20" s="3"/>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>71</v>
+        <v>22</v>
       </c>
       <c r="E21" s="3">
-        <v>3000</v>
-      </c>
-      <c r="F21" t="s" s="46">
-        <v>109</v>
-      </c>
+        <v>1000</v>
+      </c>
+      <c r="F21" s="3"/>
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F22" t="s" s="48">
-        <v>109</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="F22" s="3"/>
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="3" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="E23" s="3">
-        <v>10</v>
-      </c>
-      <c r="F23" t="s" s="50">
-        <v>109</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F23" s="3"/>
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D24" s="3" t="s">
         <v>73</v>
       </c>
-      <c r="B24" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F24" t="s" s="52">
-        <v>109</v>
-      </c>
+      <c r="E24" s="3">
+        <v>20</v>
+      </c>
+      <c r="F24" s="3"/>
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="3" t="s">
         <v>74</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="F25" t="s" s="54">
-        <v>111</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="F25" s="3"/>
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D26" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B26" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>77</v>
-      </c>
       <c r="E26" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="F26" t="s" s="57">
-        <v>109</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="F26" s="3"/>
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="B27" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="B27" s="3" t="s">
-        <v>44</v>
-      </c>
       <c r="C27" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="E27" s="3">
-        <v>10</v>
-      </c>
-      <c r="F27" t="s" s="60">
-        <v>109</v>
-      </c>
+      <c r="E27" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F27" s="3"/>
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="3" t="s">
-        <v>80</v>
+        <v>41</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>81</v>
+        <v>42</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>79</v>
+        <v>22</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="F28" t="s" s="63">
-        <v>109</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="F28" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2825,85 +2782,85 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="26.4285714285714"/>
     <col min="2" max="2" customWidth="true" width="26.2857142857143"/>
     <col min="3" max="3" customWidth="true" width="15.5714285714286"/>
-    <col min="4" max="4" customWidth="true" width="33.8571428571429"/>
+    <col min="4" max="4" customWidth="true" width="42.4285714285714"/>
     <col min="5" max="5" customWidth="true" width="70.1428571428571"/>
     <col min="6" max="6" customWidth="true" width="12.5714285714286"/>
   </cols>
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="18.75" spans="1:6">
       <c r="A1" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F2" s="3"/>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F3" s="3"/>
     </row>
     <row r="4" spans="1:6">
       <c r="A4" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>8</v>
@@ -2912,52 +2869,52 @@
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="F5" s="3"/>
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F6" s="3"/>
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E7" s="3">
         <v>10</v>
@@ -2966,34 +2923,34 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F8" s="3"/>
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E9" s="3">
         <v>10</v>
@@ -3002,106 +2959,106 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F10" s="3"/>
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E11" s="3" t="s">
         <v>87</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C11" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>89</v>
       </c>
       <c r="F11" s="3"/>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="E12" s="3" t="s">
         <v>90</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>92</v>
       </c>
       <c r="F12" s="3"/>
     </row>
     <row r="13" spans="1:6">
       <c r="A13" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="E13" s="3" t="s">
         <v>93</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>95</v>
       </c>
       <c r="F13" s="3"/>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>97</v>
+        <v>27</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>95</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F14" s="3"/>
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="E15" s="3">
         <v>5000</v>
@@ -3110,78 +3067,618 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>101</v>
+        <v>35</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>102</v>
+        <v>70</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>22</v>
       </c>
       <c r="F16" s="3"/>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="3" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>34</v>
+        <v>68</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>45</v>
+        <v>22</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>71</v>
+        <v>22</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F17" s="3"/>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="3" t="s">
-        <v>104</v>
+        <v>82</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>67</v>
+        <v>35</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>21</v>
+        <v>81</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F18" s="3"/>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="3" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F19" s="3"/>
+    </row>
+    <row r="20" spans="1:6">
+      <c r="A20" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F20" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:F25"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <cols>
+    <col min="1" max="1" customWidth="true" width="26.5714285714286"/>
+    <col min="2" max="2" customWidth="true" width="32.1428571428571"/>
+    <col min="3" max="3" customWidth="true" width="29.0"/>
+    <col min="4" max="4" customWidth="true" width="50.2857142857143"/>
+    <col min="5" max="5" customWidth="true" width="21.7142857142857"/>
+  </cols>
+  <sheetData>
+    <row r="1" s="1" customFormat="1" ht="18.75" spans="1:6">
+      <c r="A1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" t="s" s="10">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F3" t="s" s="12">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F4" t="s" s="14">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" t="s" s="16">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E6" s="3">
+        <v>3000</v>
+      </c>
+      <c r="F6" t="s" s="18">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="F7" t="s" s="20">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E8" s="3">
+        <v>3000</v>
+      </c>
+      <c r="F8" t="s" s="22">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F9" t="s" s="24">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5">
+      <c r="A10" t="s">
+        <v>103</v>
+      </c>
+      <c r="B10" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" t="s">
+        <v>104</v>
+      </c>
+      <c r="E10">
+        <v>10</v>
+      </c>
+      <c r="F10" t="s" s="26">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5">
+      <c r="A11" t="s">
+        <v>105</v>
+      </c>
+      <c r="B11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" t="s">
+        <v>46</v>
+      </c>
+      <c r="D11" t="s">
+        <v>104</v>
+      </c>
+      <c r="E11" t="s">
+        <v>22</v>
+      </c>
+      <c r="F11" t="s" s="28">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5">
+      <c r="A12" t="s">
+        <v>49</v>
+      </c>
+      <c r="B12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D12" t="s">
+        <v>106</v>
+      </c>
+      <c r="E12" t="s">
+        <v>22</v>
+      </c>
+      <c r="F12" t="s" s="30">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5">
+      <c r="A13" t="s">
+        <v>107</v>
+      </c>
+      <c r="B13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" t="s">
+        <v>46</v>
+      </c>
+      <c r="D13" t="s">
+        <v>108</v>
+      </c>
+      <c r="E13">
+        <v>10</v>
+      </c>
+      <c r="F13" t="s" s="32">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5">
+      <c r="A14" t="s">
+        <v>85</v>
+      </c>
+      <c r="B14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" t="s">
+        <v>46</v>
+      </c>
+      <c r="D14" t="s">
+        <v>108</v>
+      </c>
+      <c r="E14" t="s">
+        <v>87</v>
+      </c>
+      <c r="F14" t="s" s="34">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5">
+      <c r="A15" t="s">
+        <v>88</v>
+      </c>
+      <c r="B15" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D15" t="s">
+        <v>109</v>
+      </c>
+      <c r="E15" t="s">
+        <v>90</v>
+      </c>
+      <c r="F15" t="s" s="36">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5">
+      <c r="A16" t="s">
+        <v>91</v>
+      </c>
+      <c r="B16" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" t="s">
+        <v>110</v>
+      </c>
+      <c r="E16" t="s">
+        <v>111</v>
+      </c>
+      <c r="F16" t="s" s="38">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5">
+      <c r="A17" t="s">
+        <v>112</v>
+      </c>
+      <c r="B17" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" t="s">
+        <v>46</v>
+      </c>
+      <c r="D17" t="s">
+        <v>113</v>
+      </c>
+      <c r="E17">
+        <v>10</v>
+      </c>
+      <c r="F17" t="s" s="40">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5">
+      <c r="A18" t="s">
+        <v>114</v>
+      </c>
+      <c r="B18" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" t="s">
+        <v>46</v>
+      </c>
+      <c r="D18" t="s">
+        <v>113</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="F18" t="s" s="42">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5">
+      <c r="A19" t="s">
+        <v>116</v>
+      </c>
+      <c r="B19" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" t="s">
+        <v>46</v>
+      </c>
+      <c r="D19" t="s">
+        <v>117</v>
+      </c>
+      <c r="E19">
+        <v>10</v>
+      </c>
+      <c r="F19" t="s" s="44">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5">
+      <c r="A20" t="s">
+        <v>118</v>
+      </c>
+      <c r="B20" t="s">
+        <v>26</v>
+      </c>
+      <c r="C20" t="s">
+        <v>46</v>
+      </c>
+      <c r="D20" t="s">
+        <v>117</v>
+      </c>
+      <c r="E20">
+        <v>9876576576</v>
+      </c>
+      <c r="F20" t="s" s="46">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5">
+      <c r="A21" t="s">
+        <v>119</v>
+      </c>
+      <c r="B21" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" t="s">
+        <v>46</v>
+      </c>
+      <c r="D21" t="s">
+        <v>120</v>
+      </c>
+      <c r="E21" t="s">
+        <v>121</v>
+      </c>
+      <c r="F21" t="s" s="48">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5">
+      <c r="A22" t="s">
+        <v>122</v>
+      </c>
+      <c r="B22" t="s">
+        <v>26</v>
+      </c>
+      <c r="C22" t="s">
+        <v>46</v>
+      </c>
+      <c r="D22" t="s">
+        <v>123</v>
+      </c>
+      <c r="E22" t="s">
+        <v>124</v>
+      </c>
+      <c r="F22" t="s" s="50">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5">
+      <c r="A23" t="s">
+        <v>125</v>
+      </c>
+      <c r="B23" t="s">
+        <v>126</v>
+      </c>
+      <c r="C23" t="s">
+        <v>46</v>
+      </c>
+      <c r="D23" t="s">
+        <v>127</v>
+      </c>
+      <c r="E23" t="s">
+        <v>22</v>
+      </c>
+      <c r="F23" t="s" s="52">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5">
+      <c r="A24" t="s">
+        <v>128</v>
+      </c>
+      <c r="B24" t="s">
+        <v>35</v>
+      </c>
+      <c r="C24" t="s">
+        <v>46</v>
+      </c>
+      <c r="D24" t="s">
+        <v>129</v>
+      </c>
+      <c r="E24" t="s">
+        <v>22</v>
+      </c>
+      <c r="F24" t="s" s="54">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5">
+      <c r="A25" t="s">
+        <v>98</v>
+      </c>
+      <c r="B25" t="s">
+        <v>35</v>
+      </c>
+      <c r="C25" t="s">
+        <v>46</v>
+      </c>
+      <c r="D25" t="s">
+        <v>70</v>
+      </c>
+      <c r="E25" t="s">
+        <v>22</v>
+      </c>
+      <c r="F25" t="s" s="56">
+        <v>131</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E18" r:id="rId1" display="ydaa@gmail.com"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>